<commit_message>
Match Page_Liberman/groups.xlsx styling to the reference template
The user provided a template groups.xlsx showing the expected design:
sheet named "Groups" (not the default "Sheet1"), a bold white-on-navy
(#2E4057) centered header row at 14pt, 14pt wrapped/vertically-centered
body cells, and column widths 55/55/20 for Group Name/URL/Category.
The previous plain pandas.to_excel() output had none of that. Content
(all 116 categorized groups) is unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkU5YgS7am2HLxSqW6xu6F
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Groups" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+        <bgColor rgb="002E4057"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +60,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,1991 +435,1996 @@
   </sheetPr>
   <dimension ref="A1:C117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Group Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Нетания новости, общение, реклама</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/4073882449503859/</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Нетания</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Нетания</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1743633072506859/</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Нетания по-русски ❤️🇮🇱</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1684305088524622/</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Нетания_ОбО!ВсЕм!</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1231051221054799/</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Нетания: мероприятия, концерты, спектакли</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/netanyaevents/</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>נתניה-Нетания</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/712343903309453/</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Нетания | Израиль 🇮🇱🧡</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/netanyacity/</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Нетания на ладони</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/334095483729769/</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Нетания Шароновна / Netanya</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/208813546191502/</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>русская нетания</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/173461537349043/</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Нетания Сегодня: реклама, новости</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/666785797696690/</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Нетания, все и обо всем</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/421665435355685/</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Наша Нетания ❤️</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/304113246920348/</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Русская Нетания - Наш Дом</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1778292855801429/</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Русскоязычная Нетания 🇮🇱❤️</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/525264616838990/</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Деловые люди Нетании и не только....</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/541143452739091/</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Натания по русски</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/2848977978715762/</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Русскоговорящая Нетания</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/238775562226467/</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Голос Нетании</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/3200787340162262/</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Израиль - русскоязычные в Нетании</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/246775123870069/</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Моя Нетания - репатриация в Израиль</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/323658861172331/</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Сарафанное радио📟 Нетания</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/103503909984606/</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>НАШ ДОМ НЕТАНИЯ -OUR HOME NETANYA</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/25856052963999179/</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Нетания Доска бесплатных объявлений</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1181923921909900/</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Нетания - Доска полезных объявлений- ADS board Netanya - ישראל נתניה למכירה</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/netanya770/</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>БЕСЕДКА НЕТАНИИ</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/341111022987984/</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Нетания - Доска объявлений</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/25398870063142380/</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Нетания /Русскоязычная улица</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/BaraholkaNetaniya/</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Нетания по-русски - город Нетания - עיר נתניה</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/netanya.gorod/</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Нетания – Объявления | Общение | Бизнес</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/netanya.ad/</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Светская Нетания</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/651759856475660/</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Нетания 🇮🇱 Объявления 🇮🇱 Реклама</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/852324055883632/</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Русская Нетания</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/555945731109923/</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Нетания-наш город</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1103306336387064/</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Нетания</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Ашкелон. Израиль</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1228605825882224/</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Ashkelon.ru - אשקלון - Ашкелон</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashkelon.ru/</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Ашкелон- объявления, реклама и просто общение</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1237518529768192/</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Ашкелон #1 first</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/3058346161130314/</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Ашкелон - одна община</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/734328373706580/</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>город Ашкелон</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1524587834528066/</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>I LOVE ASHKELON - Я ЛЮБЛЮ АШКЕЛОН</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/706045636447077/</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>ашкелон</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1067722477428825/</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Ашкелонцы</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/437100913513873/</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Ашкелон - наш дом</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/MyHomeAshkelon/</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Ашкелон</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/GorodAshkelon/</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>АШКЕЛОН - городские новости</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/486181258214801/</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Ашкелон - ashkelonInfo.com</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashkeloninfo/</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Ашкелон по-русски ❤️🇮🇱</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/924731324314669/</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Ашкелон доска объявлений</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/139257533420072/</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Наш Дом Ашкелон</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1751090975126801/</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Ашкелон IL</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/143797022986144/</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Ашкелон сегодня אשקלון היום</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1103110463184655/</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Ашкелон. Реклама и объявления.</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/5091503917615876/</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Ашкелон - Доска полезных объявлений - ADS board Ashkelon - אשקלון</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashkelo/</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Мой Ашкелон</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/740808239638867/</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Ашкелон Русская Улица.</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/129841610904536/</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Ашкелон/Русскоязычная улица</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/Baraholka.Ashkelon/</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Ашкелон</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/312761484323064/</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Русские в Ашкелоне</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1395611240777418/</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Русскоязычный Ашкелон</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/650947989292864/</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Только Наш Ашкелон!!!</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/292757254691194/</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Наш любимый город Ашкелон</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/890314629049162/</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Ашкелон по другому.</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1525240427701750/</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>НАШ АШКЕЛОН . אשקלון שלנו</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1802889806668923/</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Ашкелон 🇮🇱 Объявления 🇮🇱 Реклама</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/3157642451114655/</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Ашкелон – Объявления | Общение | Бизнес</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashkelon.ads/</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Ашкелон по-русски - город Ашкелон - עיר אשקלון‏</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashkelon.gorod/</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Ашкелон и ашкелонцы</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/259939794657546/</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Доска объявлений города Ашкелон</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/100148610341310/</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>АШКЕЛОН-ИМ Доска объявлений</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/149916475720260/</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>Ашкелон для всех.</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/500814293451436/</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>Ашкелон по - русски</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/447983335961418/</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>АШКЕЛОН FOREVER</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1835042423479726/</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Ашкелон</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>Ашдод /Русская улица 🇮🇱</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashdod.russian/</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>Ашдод - по русски 2</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/336966036742161/</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>Ашдод по-русски אשדוד ברוסית</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1897984290505870/</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>Ашдод | אשדוד</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashdodmybestcity/</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>Ашдод по-русски ❤️ 🇮🇱</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1122362147806495/</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>Ашдод - Реклама</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/775901490069338/</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>✏ Ашдод /Русскоязычная улица</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/JobsAshdodRus/</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>Ашдод реклама</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1872285036226649/</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>Алия в Ашдод (Департамент абсорбции)</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/473228599548916/</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>Наш Ашдод</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/169769053100290/</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>Новости Ашдода - חדשות אשדוד</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1631303936950549/</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>Только Ашдод..</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/300108923661072/</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>Ашдод אשדוד</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/207935266455918/</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Ашдод-Ашкелон - Доска объявлений</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1995858181146645/</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>ASHDOD.RU город Ашдод</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashdod/</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>Ашдод - норм город ❤</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/616544882296990/</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>Ашдод по-русски</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/3133116813585917/</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
         <is>
           <t>Ашдод - наш город</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashdodmycity1/</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>Услуги: Ашдод, Ашкелон и окресности</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/ashkelonissafe/</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>Ашдод соседи</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/723912507627072/</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>Ашдод - доска полезных объявлений - ADS board Ashdod - אשדוד</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/434424782108297/</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>Ашдод доска объявлений</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1937391069844144/</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="2" t="inlineStr">
         <is>
           <t>Ашдод 🇮🇱 Объявления 🇮🇱 Реклама</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/338738746724298/</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Ашдод</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/cityashdod/</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="2" t="inlineStr">
         <is>
           <t>Ашдод - мой город</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/2429295583755176/</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="2" t="inlineStr">
         <is>
           <t>Ашдод По русски</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/230956371485298/</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="2" t="inlineStr">
         <is>
           <t>Ашдод русская улица ♥️</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/BaraholkaRusAshdod/</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="A102" s="2" t="inlineStr">
         <is>
           <t>Ашдод - это мы / אשדוד / Аshdod</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B102" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/361676425582140/</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t>Ашдод /Русская улица 🇮🇱</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/3283744275088722/</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
+      <c r="A104" s="2" t="inlineStr">
         <is>
           <t>Возвращаем Ашдод Ашдодцам💪💪💪</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/181786669083374/</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="2" t="inlineStr">
         <is>
           <t>Ашдод НАШ ДОМ по-русски</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/592156520977381/</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="2" t="inlineStr">
         <is>
           <t>Ашдод</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
+      <c r="A106" s="2" t="inlineStr">
         <is>
           <t>Сдерот по-русски</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B106" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/148690859079291/</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C106" s="2" t="inlineStr">
         <is>
           <t>Сдерот</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
+      <c r="A107" s="2" t="inlineStr">
         <is>
           <t>доМой</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B107" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/beitenu/</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C107" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
+      <c r="A108" s="2" t="inlineStr">
         <is>
           <t>Новости НДИ - группа сторонников</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B108" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/israelbeyteynu/</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C108" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
+      <c r="A109" s="2" t="inlineStr">
         <is>
           <t>Это наша страна © זו ארצנו</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B109" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/398730290292883/</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C109" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>ИЗРАИЛЬ ПРАВый !!! ©</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/503947849780498/</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>Группа «eXpert»</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/exprtgroup/</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
+      <c r="A112" s="2" t="inlineStr">
         <is>
           <t>Израиль - жизнь и события</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B112" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/israelnewsandoccasions/</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
+      <c r="A113" s="2" t="inlineStr">
         <is>
           <t>Я люблю Израиль</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/isroe/</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>Время Перемен</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/vremya.peremen/</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C114" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>Поддержи Израиль</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/supisrael/</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C115" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>Народ и Страна</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1248083958701234/</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C116" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>Он должен уйти!</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/1575902792579625/</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
         </is>

</xml_diff>

<commit_message>
Mark 3 confirmed groups Error_NoPostField, duplicate 14 as Тест
User manually verified these three Ashdod groups genuinely can't be
posted to, so they're now Error_NoPostField and will be skipped by
SKIP_CATEGORY going forward:
- Ашдод - наш город
- Ашдод - мой город
- Возвращаем Ашдод Ашдодцам

The other 14 groups that failed with a plain timeout in today's run
are duplicated under a new "Тест" category (originals kept under
Ашдод) so they can be re-run specifically on the updated script
(real click + longer timeout) to check whether that was genuine
account slowdown or the click/focus bug, without re-running the
whole Ашдод category.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkU5YgS7am2HLxSqW6xu6F
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Ашдод</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Ашдод</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Ашдод</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -2427,6 +2427,244 @@
       <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Политика</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод реклама</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1872285036226649/</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Алия в Ашдод (Департамент абсорбции)</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/473228599548916/</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Новости Ашдода - חדשות אשדוד</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1631303936950549/</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Только Ашдод..</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/300108923661072/</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод אשדוד</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/207935266455918/</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод-Ашкелон - Доска объявлений</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1995858181146645/</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>ASHDOD.RU город Ашдод</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/ashdod/</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод - норм город ❤</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/616544882296990/</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод по-русски</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/3133116813585917/</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Услуги: Ашдод, Ашкелон и окресности</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/ashkelonissafe/</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод соседи</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/723912507627072/</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод - доска полезных объявлений - ADS board Ashdod - אשדוד</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/434424782108297/</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод доска объявлений</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1937391069844144/</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Ашдод русская улица ♥️</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/BaraholkaRusAshdod/</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark 6 confirmed Ashkelon groups as Error_NoPostField for Liberman
Confirmed via a clean 33/39 run (zero timeout-type errors, only real
Error_NoPostField cases) that these groups genuinely don't let this
account post:
- Ашкелон - наш дом
- Ашкелон (GorodAshkelon)
- Ашкелон доска объявлений
- Мой Ашкелон
- НАШ АШКЕЛОН . אשקלון שלנו
- Ашкелон по - русски

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkU5YgS7am2HLxSqW6xu6F
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -1202,7 +1202,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 68 newly joined groups to Page_Liberman/groups.xlsx
Categorized by city per user's answers:
- Ашкелон: +3
- Беэр-Шева (new category): 38, including the general "Весь Юг Израиля"
  and multi-city groups assigned to their first-named city
- Кирьят Гат (new category): 8
- Нетивот (new category): 5
- Офаким (new category): 5
- Сдерот: +6, including two multi-city groups assigned here as their
  first-named city
- Политика: +1 ("Я русскоязычный израильтянин", general/no city)
- Left uncategorized (blank) per instruction: Кирьят Ям, Кирьят Оно
  (one group each, not enough for their own category yet)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkU5YgS7am2HLxSqW6xu6F
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2668,6 +2668,1154 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон - объявления</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/422043400438517/</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон - Доска обьявлений бесплатно</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/471399918243435/</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон. Реклама..</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2013227682251370/</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Ашкелон</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Беер-Шева на Русском</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1759982527596825/</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Интресное в Беэр Шеве на юге Израиля и другие новости</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/154106369975405/</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева юг Израиля и другие новости</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/141596652578472/</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Беер-шева.ru Новости юга Израиля</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1494682433908767/</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева и Юг - работа</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2704432896396343/</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>КРУГ ДРУЗЕЙ БЕЕР ШЕВА</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1129509880504643/</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-шева и негев, Будьте как Дома!</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1076500926302328/</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева Онлайн</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/955891061192257/</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева - Доска полезных объявлений - ADS board Beer Sheva - באר שבע</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/mybeersheva/</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева. Израиль</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/647623481002896/</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева - Жемчужина Негева</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/121321788486479/</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Доска объявлений Беер-Шева</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/312503512735671/</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева_ОбО!ВсЕм!</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/606972704227133/</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева по-русски ❤️🇮🇱</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1701086430170977/</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Беэр шева реклама</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/600074297129761/</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева /Русскоязычная улица 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/beersheva.rus/</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Беер-Шева - Доска объявлений</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1079488720984819/</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Беер-шева на русском</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/769207001226730/</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева » Доска объявлений Израиля</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/BeershebaBoard/</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева,Негев и весь Израиль.</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2340185702926960/</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>Русскоязычная Беэр Шева</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/769112478734041/</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>•Наша Беэр-Шева•</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1862667157336991/</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-шева_Израиль # Русскоязычный 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2468457136763424/</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Беер-шева</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/503246759879321/</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева на ладони</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/331030170690700/</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева по-русски</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/293926897770497/</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Беэр Шева по-русски - Беэр Шева - עיר באר שבע</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/beersheva.gorod/</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева – Объявления | Новости | Общение | Бизнес</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/Beersheba.ads/</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>юг,беер шева.</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/227342391341468/</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>Беэр шева и юг Израиля - ты не один! ❤️❤️❤️</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/696712835346644/</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева и юг Израиля</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/570772640009376/</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева 🇮🇱 Объявления 🇮🇱 Реклама</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/284808827132300/</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>БЕЕР-ШЕВА❤️МЫ ВМЕСТЕ🇮🇱</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/beershevasale1/</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>Доска обьявлений Беэр Шева.</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/BeerSheba100/</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева и Негев. Взаимопомощь.</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/beersheva.negev.ru/</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева и Негев, мы вместе!</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/BeerShevaTogetherRu/</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>Весь Юг Израиля</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/786924545196703/</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева и Негев (Юг - Ашдод, Ашкелон, Димона, Сдерот, Офаким, Нетивот...)</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/negev.Israel/</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Беэр-Шева</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>НОВОСТИ КИРЬЯТ- ГАТА.</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/167048847479991/</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>Что? Где? Почём? - Кирьят Гат</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/659506567722591/</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>КИРЬЯТ ГАТ – ИЗРАИЛЬ. Новости/Политика/Актуальное.</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2136038806451335/</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат по-русски - Город Кирят Гат - עיר קריית גת</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/kiryatgat.gorod/</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат по-русски ❤️🇮🇱</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/123754964934419/</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат - мы здесь живём</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/QiryatGatWeLiveHere/</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>Дежурные по Кирьят Гату</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/ondutyqiryatgat/</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят-Гат 🇮🇱 Объявления 🇮🇱 Реклама</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2835789163393075/</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Гат</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот. Израиль</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/4319257058218157/</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>нетивот</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/208433367612743/</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот. Русская улица ♥ 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/484567672191383/</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот /Русскоязычная улица 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/Netivot.rus/</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот по-русски - Город Нетивот - עיר נתיבות</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/netivot.gorod/</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Нетивот</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Офаким по-русски | אופקים ברוסית</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/532018987467880/</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Офаким</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>Новости Офакима</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/2404734573085219/</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Офаким</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Офаким /Русскоязычная улица 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/OfaqimRus/</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Офаким</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>Офаким 🇮🇱 Объявления 🇮🇱 Реклама</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1042648970058775/</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>Офаким</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Офаким по-русски - Город Офаким - עיר אופקים</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/ofakim.gorod/</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Офаким</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот, Офаким, Нетивот по-русски ❤️🇮🇱</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/156573954883476/</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот по-русски - Город Сдерот - עיר שדרות</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/sderot.gorod/</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот и Негев (Юг - Сдерот, Офаким, Нетивот, Кирьят гат...)</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/173375400654523/</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот. Русская улица ♥ 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/154348401968537/</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот 🇮🇱 Объявления 🇮🇱 Реклама</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/133278689840028/</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот /Русскоязычная улица 🇮🇱</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/SderotRus/</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>Сдерот</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>Я русскоязычный израильтянин</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1650272811683869/</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>Политика</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Ям по-русски - Город Кирьят Ям - עיר קריית ים</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/kiryatyam.gorod/</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>Кирьят Оно по-русски - Город Кирьят Оно - עיר קריית אונו</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/kiryatono.gorod/</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark 4 confirmed Netanya groups Error_NoPostField, duplicate 10 as Тест
From today's 34-group Netanya run on the old (send_keys) script
version: 4 groups genuinely never open the post field (confirmed
Error_NoPostField, same as a human would see) and are now permanently
skipped via SKIP_CATEGORY:
- Русская Нетания - Наш Дом
- Израиль - русскоязычные в Нетании
- Нетания - Доска полезных объявлений- ADS board Netanya
- Нетания /Русскоязычная улица

The other 10 groups failed with a plain Error (timeout) partway
through the run -- duplicated into the Тест category (originals kept
under Нетания) so they can be re-run specifically on the CDP-based
file upload version to compare against the send_keys mechanism.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkU5YgS7am2HLxSqW6xu6F
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C199"/>
+  <dimension ref="A1:C209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Нетания</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Нетания</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Нетания</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Нетания</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -3815,6 +3815,176 @@
         </is>
       </c>
       <c r="C199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>НАШ ДОМ НЕТАНИЯ -OUR HOME NETANYA</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/25856052963999179/</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>Нетания Доска бесплатных объявлений</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1181923921909900/</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>БЕСЕДКА НЕТАНИИ</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/341111022987984/</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Нетания - Доска объявлений</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/25398870063142380/</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Нетания по-русски - город Нетания - עיר נתניה</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/netanya.gorod/</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Нетания – Объявления | Общение | Бизнес</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/netanya.ad/</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Светская Нетания</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/651759856475660/</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Нетания 🇮🇱 Объявления 🇮🇱 Реклама</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/852324055883632/</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Русская Нетания</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/555945731109923/</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>Нетания-наш город</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1103306336387064/</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Тест</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Split the 10 Netanya retest groups into a separate Тест 2 category
Keeps the original Тест (14 Ashdod groups) and the new Netanya batch
separate rather than merged, so each retest run can be scoped to one
batch at a time.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GkU5YgS7am2HLxSqW6xu6F
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -3829,7 +3829,7 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Тест</t>
+          <t>Тест 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark 2 more confirmed-bad groups as Error_NoPostField
Both failed with Error_NoPostField in two clean full-category runs
(Ashdod 27/28, Ashkelon 35/36) using the new attach-media-first + retry
logic -- no sign of composer degradation in either run, just these two
groups' composer never opening (group likely closed/restricted):
- Ашдод /Русскоязычная улица
- Ашкелон/Русскоязычная улица
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -1423,7 +1423,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Ашкелон</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Ашдод</t>
+          <t>Error_NoPostField</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge 17 Бат Ям groups added locally on the Windows machine
Found while reconciling before converting the Windows project folder to
a git clone: the user's local groups.xlsx had gained a "Бат Ям" category
(17 groups) added directly on that machine after the last sync here on
Oct 10, never sent back. The repo's copy was otherwise ahead (7 more
confirmed Error_NoPostField markings from since-then runs) with no other
divergence. Merged the 17 new rows in on top of the repo's version
rather than letting the upcoming git checkout silently overwrite and
lose them.
</commit_message>
<xml_diff>
--- a/Page_Liberman/groups.xlsx
+++ b/Page_Liberman/groups.xlsx
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +117,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -484,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D255"/>
+  <dimension ref="A1:D272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5595,6 +5601,346 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" s="6" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" s="7" t="inlineStr">
+        <is>
+          <t>Бат Ям по-русски - Город Бат Ям - עיר בת ים</t>
+        </is>
+      </c>
+      <c r="C256" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/batyam.gorod/</t>
+        </is>
+      </c>
+      <c r="D256" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="6" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" s="7" t="inlineStr">
+        <is>
+          <t>Бат ям новости, общение, реклама</t>
+        </is>
+      </c>
+      <c r="C257" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/453511942069355/</t>
+        </is>
+      </c>
+      <c r="D257" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="6" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" s="7" t="inlineStr">
+        <is>
+          <t>Бат-Ям – Объявления | Общение | Бизнес</t>
+        </is>
+      </c>
+      <c r="C258" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/batyam.ad/</t>
+        </is>
+      </c>
+      <c r="D258" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="6" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" s="7" t="inlineStr">
+        <is>
+          <t>Бат-Ям /Русская улица.Гуш-Дан — Бат-Ям, Тель-Авив — Яффо, Холон, Рамат-Ган</t>
+        </is>
+      </c>
+      <c r="C259" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/233260368318381/</t>
+        </is>
+      </c>
+      <c r="D259" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="6" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" s="7" t="inlineStr">
+        <is>
+          <t>Бат-Ям 🇮🇱 Объявления 🇮🇱 Реклама</t>
+        </is>
+      </c>
+      <c r="C260" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/242295524936952/</t>
+        </is>
+      </c>
+      <c r="D260" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="6" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" s="7" t="inlineStr">
+        <is>
+          <t>Бат ям жизнь города 🏙</t>
+        </is>
+      </c>
+      <c r="C261" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/kleobatyam/</t>
+        </is>
+      </c>
+      <c r="D261" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" s="7" t="inlineStr">
+        <is>
+          <t>НОВЫЙ БАТ ЯМ</t>
+        </is>
+      </c>
+      <c r="C262" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/newbatyam/</t>
+        </is>
+      </c>
+      <c r="D262" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="6" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" s="7" t="inlineStr">
+        <is>
+          <t>Бат Ям - Доска полезных объявлений- ADS board Bat Yam - ישראל בת ים</t>
+        </is>
+      </c>
+      <c r="C263" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/3215330658684975/</t>
+        </is>
+      </c>
+      <c r="D263" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="6" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" s="7" t="inlineStr">
+        <is>
+          <t>Бат-Ям вся реклама в одном месте</t>
+        </is>
+      </c>
+      <c r="C264" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/940641719347331/</t>
+        </is>
+      </c>
+      <c r="D264" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="6" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" s="7" t="inlineStr">
+        <is>
+          <t>Бат Ям / Русская Улица 🇮🇱</t>
+        </is>
+      </c>
+      <c r="C265" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1580441979019302/</t>
+        </is>
+      </c>
+      <c r="D265" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="6" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" s="7" t="inlineStr">
+        <is>
+          <t>Бат Ям / Русская Улица 🇮🇱</t>
+        </is>
+      </c>
+      <c r="C266" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/578917473330175/</t>
+        </is>
+      </c>
+      <c r="D266" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="6" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" s="7" t="inlineStr">
+        <is>
+          <t>Русскоязычные специалисты в г. Бат-Ям</t>
+        </is>
+      </c>
+      <c r="C267" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/334863070705655/</t>
+        </is>
+      </c>
+      <c r="D267" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="6" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" s="7" t="inlineStr">
+        <is>
+          <t>Бат-Ям - Доска объявлений</t>
+        </is>
+      </c>
+      <c r="C268" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/898735946038038/</t>
+        </is>
+      </c>
+      <c r="D268" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="6" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" s="7" t="inlineStr">
+        <is>
+          <t>БАТ-ЯМ и соседи (Гуш-Дан 🇮🇱)</t>
+        </is>
+      </c>
+      <c r="C269" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/gushdanrus/</t>
+        </is>
+      </c>
+      <c r="D269" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="6" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" s="7" t="inlineStr">
+        <is>
+          <t>Бат Ям по-русски ❤️🇮🇱</t>
+        </is>
+      </c>
+      <c r="C270" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/473713946160027/</t>
+        </is>
+      </c>
+      <c r="D270" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="6" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" s="7" t="inlineStr">
+        <is>
+          <t>Бат ям - Холон реклама</t>
+        </is>
+      </c>
+      <c r="C271" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/965950493555492/</t>
+        </is>
+      </c>
+      <c r="D271" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="6" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" s="7" t="inlineStr">
+        <is>
+          <t>Бат - ям. 24/7 Бесплатная доска объявлений</t>
+        </is>
+      </c>
+      <c r="C272" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/708040567155047/</t>
+        </is>
+      </c>
+      <c r="D272" s="6" t="inlineStr">
+        <is>
+          <t>Бат Ям</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>